<commit_message>
Add Ashish Arya (Momo Box) and Pushpendra (Koby's) with photos
- Ashish Arya added to end of The Momo Box group (photo attached)
- Pushpendra added to end of Koby's group (photo attached)
- Other details (Emp ID, contact, Aadhaar) left blank for later
- Total employees now 67; S.No renumbered 1-67
</commit_message>
<xml_diff>
--- a/Azimuth Food Street Staff FRS details 29sept.xlsx
+++ b/Azimuth Food Street Staff FRS details 29sept.xlsx
@@ -1250,664 +1250,714 @@
       <row>41</row>
       <rowOff>0</rowOff>
     </from>
+    <ext cx="628650" cy="838200"/>
+    <pic>
+      <nvPicPr>
+        <cNvPr id="39" name="Image 39" descr="Picture"/>
+        <cNvPicPr/>
+      </nvPicPr>
+      <blipFill>
+        <a:blip cstate="print" r:embed="rId39"/>
+        <a:stretch>
+          <a:fillRect/>
+        </a:stretch>
+      </blipFill>
+      <spPr>
+        <a:prstGeom prst="rect"/>
+      </spPr>
+    </pic>
+    <clientData/>
+  </oneCellAnchor>
+  <oneCellAnchor>
+    <from>
+      <col>5</col>
+      <colOff>0</colOff>
+      <row>42</row>
+      <rowOff>0</rowOff>
+    </from>
     <ext cx="704850" cy="838200"/>
     <pic>
       <nvPicPr>
-        <cNvPr id="39" name="Image 39" descr="Picture"/>
-        <cNvPicPr/>
-      </nvPicPr>
-      <blipFill>
-        <a:blip cstate="print" r:embed="rId39"/>
-        <a:stretch>
-          <a:fillRect/>
-        </a:stretch>
-      </blipFill>
-      <spPr>
-        <a:prstGeom prst="rect"/>
-      </spPr>
-    </pic>
-    <clientData/>
-  </oneCellAnchor>
-  <oneCellAnchor>
-    <from>
-      <col>5</col>
-      <colOff>0</colOff>
-      <row>42</row>
+        <cNvPr id="40" name="Image 40" descr="Picture"/>
+        <cNvPicPr/>
+      </nvPicPr>
+      <blipFill>
+        <a:blip cstate="print" r:embed="rId40"/>
+        <a:stretch>
+          <a:fillRect/>
+        </a:stretch>
+      </blipFill>
+      <spPr>
+        <a:prstGeom prst="rect"/>
+      </spPr>
+    </pic>
+    <clientData/>
+  </oneCellAnchor>
+  <oneCellAnchor>
+    <from>
+      <col>5</col>
+      <colOff>0</colOff>
+      <row>43</row>
       <rowOff>0</rowOff>
     </from>
     <ext cx="685800" cy="838200"/>
     <pic>
       <nvPicPr>
-        <cNvPr id="40" name="Image 40" descr="Picture"/>
-        <cNvPicPr/>
-      </nvPicPr>
-      <blipFill>
-        <a:blip cstate="print" r:embed="rId40"/>
-        <a:stretch>
-          <a:fillRect/>
-        </a:stretch>
-      </blipFill>
-      <spPr>
-        <a:prstGeom prst="rect"/>
-      </spPr>
-    </pic>
-    <clientData/>
-  </oneCellAnchor>
-  <oneCellAnchor>
-    <from>
-      <col>5</col>
-      <colOff>0</colOff>
-      <row>43</row>
+        <cNvPr id="41" name="Image 41" descr="Picture"/>
+        <cNvPicPr/>
+      </nvPicPr>
+      <blipFill>
+        <a:blip cstate="print" r:embed="rId41"/>
+        <a:stretch>
+          <a:fillRect/>
+        </a:stretch>
+      </blipFill>
+      <spPr>
+        <a:prstGeom prst="rect"/>
+      </spPr>
+    </pic>
+    <clientData/>
+  </oneCellAnchor>
+  <oneCellAnchor>
+    <from>
+      <col>5</col>
+      <colOff>0</colOff>
+      <row>44</row>
       <rowOff>0</rowOff>
     </from>
     <ext cx="838200" cy="838200"/>
     <pic>
       <nvPicPr>
-        <cNvPr id="41" name="Image 41" descr="Picture"/>
-        <cNvPicPr/>
-      </nvPicPr>
-      <blipFill>
-        <a:blip cstate="print" r:embed="rId41"/>
-        <a:stretch>
-          <a:fillRect/>
-        </a:stretch>
-      </blipFill>
-      <spPr>
-        <a:prstGeom prst="rect"/>
-      </spPr>
-    </pic>
-    <clientData/>
-  </oneCellAnchor>
-  <oneCellAnchor>
-    <from>
-      <col>5</col>
-      <colOff>0</colOff>
-      <row>44</row>
+        <cNvPr id="42" name="Image 42" descr="Picture"/>
+        <cNvPicPr/>
+      </nvPicPr>
+      <blipFill>
+        <a:blip cstate="print" r:embed="rId42"/>
+        <a:stretch>
+          <a:fillRect/>
+        </a:stretch>
+      </blipFill>
+      <spPr>
+        <a:prstGeom prst="rect"/>
+      </spPr>
+    </pic>
+    <clientData/>
+  </oneCellAnchor>
+  <oneCellAnchor>
+    <from>
+      <col>5</col>
+      <colOff>0</colOff>
+      <row>45</row>
       <rowOff>0</rowOff>
     </from>
     <ext cx="466725" cy="838200"/>
     <pic>
       <nvPicPr>
-        <cNvPr id="42" name="Image 42" descr="Picture"/>
-        <cNvPicPr/>
-      </nvPicPr>
-      <blipFill>
-        <a:blip cstate="print" r:embed="rId42"/>
-        <a:stretch>
-          <a:fillRect/>
-        </a:stretch>
-      </blipFill>
-      <spPr>
-        <a:prstGeom prst="rect"/>
-      </spPr>
-    </pic>
-    <clientData/>
-  </oneCellAnchor>
-  <oneCellAnchor>
-    <from>
-      <col>5</col>
-      <colOff>0</colOff>
-      <row>45</row>
+        <cNvPr id="43" name="Image 43" descr="Picture"/>
+        <cNvPicPr/>
+      </nvPicPr>
+      <blipFill>
+        <a:blip cstate="print" r:embed="rId43"/>
+        <a:stretch>
+          <a:fillRect/>
+        </a:stretch>
+      </blipFill>
+      <spPr>
+        <a:prstGeom prst="rect"/>
+      </spPr>
+    </pic>
+    <clientData/>
+  </oneCellAnchor>
+  <oneCellAnchor>
+    <from>
+      <col>5</col>
+      <colOff>0</colOff>
+      <row>46</row>
       <rowOff>0</rowOff>
     </from>
     <ext cx="466725" cy="838200"/>
     <pic>
       <nvPicPr>
-        <cNvPr id="43" name="Image 43" descr="Picture"/>
-        <cNvPicPr/>
-      </nvPicPr>
-      <blipFill>
-        <a:blip cstate="print" r:embed="rId43"/>
-        <a:stretch>
-          <a:fillRect/>
-        </a:stretch>
-      </blipFill>
-      <spPr>
-        <a:prstGeom prst="rect"/>
-      </spPr>
-    </pic>
-    <clientData/>
-  </oneCellAnchor>
-  <oneCellAnchor>
-    <from>
-      <col>5</col>
-      <colOff>0</colOff>
-      <row>46</row>
+        <cNvPr id="44" name="Image 44" descr="Picture"/>
+        <cNvPicPr/>
+      </nvPicPr>
+      <blipFill>
+        <a:blip cstate="print" r:embed="rId44"/>
+        <a:stretch>
+          <a:fillRect/>
+        </a:stretch>
+      </blipFill>
+      <spPr>
+        <a:prstGeom prst="rect"/>
+      </spPr>
+    </pic>
+    <clientData/>
+  </oneCellAnchor>
+  <oneCellAnchor>
+    <from>
+      <col>5</col>
+      <colOff>0</colOff>
+      <row>47</row>
       <rowOff>0</rowOff>
     </from>
     <ext cx="628650" cy="838200"/>
     <pic>
       <nvPicPr>
-        <cNvPr id="44" name="Image 44" descr="Picture"/>
-        <cNvPicPr/>
-      </nvPicPr>
-      <blipFill>
-        <a:blip cstate="print" r:embed="rId44"/>
-        <a:stretch>
-          <a:fillRect/>
-        </a:stretch>
-      </blipFill>
-      <spPr>
-        <a:prstGeom prst="rect"/>
-      </spPr>
-    </pic>
-    <clientData/>
-  </oneCellAnchor>
-  <oneCellAnchor>
-    <from>
-      <col>5</col>
-      <colOff>0</colOff>
-      <row>47</row>
+        <cNvPr id="45" name="Image 45" descr="Picture"/>
+        <cNvPicPr/>
+      </nvPicPr>
+      <blipFill>
+        <a:blip cstate="print" r:embed="rId45"/>
+        <a:stretch>
+          <a:fillRect/>
+        </a:stretch>
+      </blipFill>
+      <spPr>
+        <a:prstGeom prst="rect"/>
+      </spPr>
+    </pic>
+    <clientData/>
+  </oneCellAnchor>
+  <oneCellAnchor>
+    <from>
+      <col>5</col>
+      <colOff>0</colOff>
+      <row>48</row>
       <rowOff>0</rowOff>
     </from>
     <ext cx="466725" cy="838200"/>
     <pic>
       <nvPicPr>
-        <cNvPr id="45" name="Image 45" descr="Picture"/>
-        <cNvPicPr/>
-      </nvPicPr>
-      <blipFill>
-        <a:blip cstate="print" r:embed="rId45"/>
-        <a:stretch>
-          <a:fillRect/>
-        </a:stretch>
-      </blipFill>
-      <spPr>
-        <a:prstGeom prst="rect"/>
-      </spPr>
-    </pic>
-    <clientData/>
-  </oneCellAnchor>
-  <oneCellAnchor>
-    <from>
-      <col>5</col>
-      <colOff>0</colOff>
-      <row>48</row>
+        <cNvPr id="46" name="Image 46" descr="Picture"/>
+        <cNvPicPr/>
+      </nvPicPr>
+      <blipFill>
+        <a:blip cstate="print" r:embed="rId46"/>
+        <a:stretch>
+          <a:fillRect/>
+        </a:stretch>
+      </blipFill>
+      <spPr>
+        <a:prstGeom prst="rect"/>
+      </spPr>
+    </pic>
+    <clientData/>
+  </oneCellAnchor>
+  <oneCellAnchor>
+    <from>
+      <col>5</col>
+      <colOff>0</colOff>
+      <row>49</row>
       <rowOff>0</rowOff>
     </from>
     <ext cx="847725" cy="838200"/>
     <pic>
       <nvPicPr>
-        <cNvPr id="46" name="Image 46" descr="Picture"/>
-        <cNvPicPr/>
-      </nvPicPr>
-      <blipFill>
-        <a:blip cstate="print" r:embed="rId46"/>
-        <a:stretch>
-          <a:fillRect/>
-        </a:stretch>
-      </blipFill>
-      <spPr>
-        <a:prstGeom prst="rect"/>
-      </spPr>
-    </pic>
-    <clientData/>
-  </oneCellAnchor>
-  <oneCellAnchor>
-    <from>
-      <col>5</col>
-      <colOff>0</colOff>
-      <row>49</row>
+        <cNvPr id="47" name="Image 47" descr="Picture"/>
+        <cNvPicPr/>
+      </nvPicPr>
+      <blipFill>
+        <a:blip cstate="print" r:embed="rId47"/>
+        <a:stretch>
+          <a:fillRect/>
+        </a:stretch>
+      </blipFill>
+      <spPr>
+        <a:prstGeom prst="rect"/>
+      </spPr>
+    </pic>
+    <clientData/>
+  </oneCellAnchor>
+  <oneCellAnchor>
+    <from>
+      <col>5</col>
+      <colOff>0</colOff>
+      <row>50</row>
       <rowOff>0</rowOff>
     </from>
     <ext cx="704850" cy="838200"/>
     <pic>
       <nvPicPr>
-        <cNvPr id="47" name="Image 47" descr="Picture"/>
-        <cNvPicPr/>
-      </nvPicPr>
-      <blipFill>
-        <a:blip cstate="print" r:embed="rId47"/>
-        <a:stretch>
-          <a:fillRect/>
-        </a:stretch>
-      </blipFill>
-      <spPr>
-        <a:prstGeom prst="rect"/>
-      </spPr>
-    </pic>
-    <clientData/>
-  </oneCellAnchor>
-  <oneCellAnchor>
-    <from>
-      <col>5</col>
-      <colOff>0</colOff>
-      <row>50</row>
+        <cNvPr id="48" name="Image 48" descr="Picture"/>
+        <cNvPicPr/>
+      </nvPicPr>
+      <blipFill>
+        <a:blip cstate="print" r:embed="rId48"/>
+        <a:stretch>
+          <a:fillRect/>
+        </a:stretch>
+      </blipFill>
+      <spPr>
+        <a:prstGeom prst="rect"/>
+      </spPr>
+    </pic>
+    <clientData/>
+  </oneCellAnchor>
+  <oneCellAnchor>
+    <from>
+      <col>5</col>
+      <colOff>0</colOff>
+      <row>51</row>
       <rowOff>0</rowOff>
     </from>
     <ext cx="685800" cy="838200"/>
     <pic>
       <nvPicPr>
-        <cNvPr id="48" name="Image 48" descr="Picture"/>
-        <cNvPicPr/>
-      </nvPicPr>
-      <blipFill>
-        <a:blip cstate="print" r:embed="rId48"/>
-        <a:stretch>
-          <a:fillRect/>
-        </a:stretch>
-      </blipFill>
-      <spPr>
-        <a:prstGeom prst="rect"/>
-      </spPr>
-    </pic>
-    <clientData/>
-  </oneCellAnchor>
-  <oneCellAnchor>
-    <from>
-      <col>5</col>
-      <colOff>0</colOff>
-      <row>51</row>
+        <cNvPr id="49" name="Image 49" descr="Picture"/>
+        <cNvPicPr/>
+      </nvPicPr>
+      <blipFill>
+        <a:blip cstate="print" r:embed="rId49"/>
+        <a:stretch>
+          <a:fillRect/>
+        </a:stretch>
+      </blipFill>
+      <spPr>
+        <a:prstGeom prst="rect"/>
+      </spPr>
+    </pic>
+    <clientData/>
+  </oneCellAnchor>
+  <oneCellAnchor>
+    <from>
+      <col>5</col>
+      <colOff>0</colOff>
+      <row>52</row>
       <rowOff>0</rowOff>
     </from>
     <ext cx="466725" cy="838200"/>
     <pic>
       <nvPicPr>
-        <cNvPr id="49" name="Image 49" descr="Picture"/>
-        <cNvPicPr/>
-      </nvPicPr>
-      <blipFill>
-        <a:blip cstate="print" r:embed="rId49"/>
-        <a:stretch>
-          <a:fillRect/>
-        </a:stretch>
-      </blipFill>
-      <spPr>
-        <a:prstGeom prst="rect"/>
-      </spPr>
-    </pic>
-    <clientData/>
-  </oneCellAnchor>
-  <oneCellAnchor>
-    <from>
-      <col>5</col>
-      <colOff>0</colOff>
-      <row>52</row>
+        <cNvPr id="50" name="Image 50" descr="Picture"/>
+        <cNvPicPr/>
+      </nvPicPr>
+      <blipFill>
+        <a:blip cstate="print" r:embed="rId50"/>
+        <a:stretch>
+          <a:fillRect/>
+        </a:stretch>
+      </blipFill>
+      <spPr>
+        <a:prstGeom prst="rect"/>
+      </spPr>
+    </pic>
+    <clientData/>
+  </oneCellAnchor>
+  <oneCellAnchor>
+    <from>
+      <col>5</col>
+      <colOff>0</colOff>
+      <row>53</row>
+      <rowOff>0</rowOff>
+    </from>
+    <ext cx="466725" cy="838200"/>
+    <pic>
+      <nvPicPr>
+        <cNvPr id="51" name="Image 51" descr="Picture"/>
+        <cNvPicPr/>
+      </nvPicPr>
+      <blipFill>
+        <a:blip cstate="print" r:embed="rId51"/>
+        <a:stretch>
+          <a:fillRect/>
+        </a:stretch>
+      </blipFill>
+      <spPr>
+        <a:prstGeom prst="rect"/>
+      </spPr>
+    </pic>
+    <clientData/>
+  </oneCellAnchor>
+  <oneCellAnchor>
+    <from>
+      <col>5</col>
+      <colOff>0</colOff>
+      <row>54</row>
       <rowOff>0</rowOff>
     </from>
     <ext cx="666750" cy="838200"/>
     <pic>
       <nvPicPr>
-        <cNvPr id="50" name="Image 50" descr="Picture"/>
-        <cNvPicPr/>
-      </nvPicPr>
-      <blipFill>
-        <a:blip cstate="print" r:embed="rId50"/>
-        <a:stretch>
-          <a:fillRect/>
-        </a:stretch>
-      </blipFill>
-      <spPr>
-        <a:prstGeom prst="rect"/>
-      </spPr>
-    </pic>
-    <clientData/>
-  </oneCellAnchor>
-  <oneCellAnchor>
-    <from>
-      <col>5</col>
-      <colOff>0</colOff>
-      <row>53</row>
+        <cNvPr id="52" name="Image 52" descr="Picture"/>
+        <cNvPicPr/>
+      </nvPicPr>
+      <blipFill>
+        <a:blip cstate="print" r:embed="rId52"/>
+        <a:stretch>
+          <a:fillRect/>
+        </a:stretch>
+      </blipFill>
+      <spPr>
+        <a:prstGeom prst="rect"/>
+      </spPr>
+    </pic>
+    <clientData/>
+  </oneCellAnchor>
+  <oneCellAnchor>
+    <from>
+      <col>5</col>
+      <colOff>0</colOff>
+      <row>55</row>
       <rowOff>0</rowOff>
     </from>
     <ext cx="628650" cy="838200"/>
     <pic>
       <nvPicPr>
-        <cNvPr id="51" name="Image 51" descr="Picture"/>
-        <cNvPicPr/>
-      </nvPicPr>
-      <blipFill>
-        <a:blip cstate="print" r:embed="rId51"/>
-        <a:stretch>
-          <a:fillRect/>
-        </a:stretch>
-      </blipFill>
-      <spPr>
-        <a:prstGeom prst="rect"/>
-      </spPr>
-    </pic>
-    <clientData/>
-  </oneCellAnchor>
-  <oneCellAnchor>
-    <from>
-      <col>5</col>
-      <colOff>0</colOff>
-      <row>54</row>
+        <cNvPr id="53" name="Image 53" descr="Picture"/>
+        <cNvPicPr/>
+      </nvPicPr>
+      <blipFill>
+        <a:blip cstate="print" r:embed="rId53"/>
+        <a:stretch>
+          <a:fillRect/>
+        </a:stretch>
+      </blipFill>
+      <spPr>
+        <a:prstGeom prst="rect"/>
+      </spPr>
+    </pic>
+    <clientData/>
+  </oneCellAnchor>
+  <oneCellAnchor>
+    <from>
+      <col>5</col>
+      <colOff>0</colOff>
+      <row>56</row>
       <rowOff>0</rowOff>
     </from>
     <ext cx="628650" cy="838200"/>
     <pic>
       <nvPicPr>
-        <cNvPr id="52" name="Image 52" descr="Picture"/>
-        <cNvPicPr/>
-      </nvPicPr>
-      <blipFill>
-        <a:blip cstate="print" r:embed="rId52"/>
-        <a:stretch>
-          <a:fillRect/>
-        </a:stretch>
-      </blipFill>
-      <spPr>
-        <a:prstGeom prst="rect"/>
-      </spPr>
-    </pic>
-    <clientData/>
-  </oneCellAnchor>
-  <oneCellAnchor>
-    <from>
-      <col>5</col>
-      <colOff>0</colOff>
-      <row>55</row>
+        <cNvPr id="54" name="Image 54" descr="Picture"/>
+        <cNvPicPr/>
+      </nvPicPr>
+      <blipFill>
+        <a:blip cstate="print" r:embed="rId54"/>
+        <a:stretch>
+          <a:fillRect/>
+        </a:stretch>
+      </blipFill>
+      <spPr>
+        <a:prstGeom prst="rect"/>
+      </spPr>
+    </pic>
+    <clientData/>
+  </oneCellAnchor>
+  <oneCellAnchor>
+    <from>
+      <col>5</col>
+      <colOff>0</colOff>
+      <row>57</row>
       <rowOff>0</rowOff>
     </from>
     <ext cx="628650" cy="838200"/>
     <pic>
       <nvPicPr>
-        <cNvPr id="53" name="Image 53" descr="Picture"/>
-        <cNvPicPr/>
-      </nvPicPr>
-      <blipFill>
-        <a:blip cstate="print" r:embed="rId53"/>
-        <a:stretch>
-          <a:fillRect/>
-        </a:stretch>
-      </blipFill>
-      <spPr>
-        <a:prstGeom prst="rect"/>
-      </spPr>
-    </pic>
-    <clientData/>
-  </oneCellAnchor>
-  <oneCellAnchor>
-    <from>
-      <col>5</col>
-      <colOff>0</colOff>
-      <row>56</row>
+        <cNvPr id="55" name="Image 55" descr="Picture"/>
+        <cNvPicPr/>
+      </nvPicPr>
+      <blipFill>
+        <a:blip cstate="print" r:embed="rId55"/>
+        <a:stretch>
+          <a:fillRect/>
+        </a:stretch>
+      </blipFill>
+      <spPr>
+        <a:prstGeom prst="rect"/>
+      </spPr>
+    </pic>
+    <clientData/>
+  </oneCellAnchor>
+  <oneCellAnchor>
+    <from>
+      <col>5</col>
+      <colOff>0</colOff>
+      <row>58</row>
       <rowOff>0</rowOff>
     </from>
     <ext cx="628650" cy="838200"/>
     <pic>
       <nvPicPr>
-        <cNvPr id="54" name="Image 54" descr="Picture"/>
-        <cNvPicPr/>
-      </nvPicPr>
-      <blipFill>
-        <a:blip cstate="print" r:embed="rId54"/>
-        <a:stretch>
-          <a:fillRect/>
-        </a:stretch>
-      </blipFill>
-      <spPr>
-        <a:prstGeom prst="rect"/>
-      </spPr>
-    </pic>
-    <clientData/>
-  </oneCellAnchor>
-  <oneCellAnchor>
-    <from>
-      <col>5</col>
-      <colOff>0</colOff>
-      <row>57</row>
+        <cNvPr id="56" name="Image 56" descr="Picture"/>
+        <cNvPicPr/>
+      </nvPicPr>
+      <blipFill>
+        <a:blip cstate="print" r:embed="rId56"/>
+        <a:stretch>
+          <a:fillRect/>
+        </a:stretch>
+      </blipFill>
+      <spPr>
+        <a:prstGeom prst="rect"/>
+      </spPr>
+    </pic>
+    <clientData/>
+  </oneCellAnchor>
+  <oneCellAnchor>
+    <from>
+      <col>5</col>
+      <colOff>0</colOff>
+      <row>59</row>
       <rowOff>0</rowOff>
     </from>
     <ext cx="476250" cy="838200"/>
     <pic>
       <nvPicPr>
-        <cNvPr id="55" name="Image 55" descr="Picture"/>
-        <cNvPicPr/>
-      </nvPicPr>
-      <blipFill>
-        <a:blip cstate="print" r:embed="rId55"/>
-        <a:stretch>
-          <a:fillRect/>
-        </a:stretch>
-      </blipFill>
-      <spPr>
-        <a:prstGeom prst="rect"/>
-      </spPr>
-    </pic>
-    <clientData/>
-  </oneCellAnchor>
-  <oneCellAnchor>
-    <from>
-      <col>5</col>
-      <colOff>0</colOff>
-      <row>58</row>
+        <cNvPr id="57" name="Image 57" descr="Picture"/>
+        <cNvPicPr/>
+      </nvPicPr>
+      <blipFill>
+        <a:blip cstate="print" r:embed="rId57"/>
+        <a:stretch>
+          <a:fillRect/>
+        </a:stretch>
+      </blipFill>
+      <spPr>
+        <a:prstGeom prst="rect"/>
+      </spPr>
+    </pic>
+    <clientData/>
+  </oneCellAnchor>
+  <oneCellAnchor>
+    <from>
+      <col>5</col>
+      <colOff>0</colOff>
+      <row>60</row>
       <rowOff>0</rowOff>
     </from>
     <ext cx="714375" cy="838200"/>
     <pic>
       <nvPicPr>
-        <cNvPr id="56" name="Image 56" descr="Picture"/>
-        <cNvPicPr/>
-      </nvPicPr>
-      <blipFill>
-        <a:blip cstate="print" r:embed="rId56"/>
-        <a:stretch>
-          <a:fillRect/>
-        </a:stretch>
-      </blipFill>
-      <spPr>
-        <a:prstGeom prst="rect"/>
-      </spPr>
-    </pic>
-    <clientData/>
-  </oneCellAnchor>
-  <oneCellAnchor>
-    <from>
-      <col>5</col>
-      <colOff>0</colOff>
-      <row>59</row>
+        <cNvPr id="58" name="Image 58" descr="Picture"/>
+        <cNvPicPr/>
+      </nvPicPr>
+      <blipFill>
+        <a:blip cstate="print" r:embed="rId58"/>
+        <a:stretch>
+          <a:fillRect/>
+        </a:stretch>
+      </blipFill>
+      <spPr>
+        <a:prstGeom prst="rect"/>
+      </spPr>
+    </pic>
+    <clientData/>
+  </oneCellAnchor>
+  <oneCellAnchor>
+    <from>
+      <col>5</col>
+      <colOff>0</colOff>
+      <row>61</row>
       <rowOff>0</rowOff>
     </from>
     <ext cx="609600" cy="838200"/>
     <pic>
       <nvPicPr>
-        <cNvPr id="57" name="Image 57" descr="Picture"/>
-        <cNvPicPr/>
-      </nvPicPr>
-      <blipFill>
-        <a:blip cstate="print" r:embed="rId57"/>
-        <a:stretch>
-          <a:fillRect/>
-        </a:stretch>
-      </blipFill>
-      <spPr>
-        <a:prstGeom prst="rect"/>
-      </spPr>
-    </pic>
-    <clientData/>
-  </oneCellAnchor>
-  <oneCellAnchor>
-    <from>
-      <col>5</col>
-      <colOff>0</colOff>
-      <row>60</row>
+        <cNvPr id="59" name="Image 59" descr="Picture"/>
+        <cNvPicPr/>
+      </nvPicPr>
+      <blipFill>
+        <a:blip cstate="print" r:embed="rId59"/>
+        <a:stretch>
+          <a:fillRect/>
+        </a:stretch>
+      </blipFill>
+      <spPr>
+        <a:prstGeom prst="rect"/>
+      </spPr>
+    </pic>
+    <clientData/>
+  </oneCellAnchor>
+  <oneCellAnchor>
+    <from>
+      <col>5</col>
+      <colOff>0</colOff>
+      <row>62</row>
       <rowOff>0</rowOff>
     </from>
     <ext cx="809625" cy="838200"/>
     <pic>
       <nvPicPr>
-        <cNvPr id="58" name="Image 58" descr="Picture"/>
-        <cNvPicPr/>
-      </nvPicPr>
-      <blipFill>
-        <a:blip cstate="print" r:embed="rId58"/>
-        <a:stretch>
-          <a:fillRect/>
-        </a:stretch>
-      </blipFill>
-      <spPr>
-        <a:prstGeom prst="rect"/>
-      </spPr>
-    </pic>
-    <clientData/>
-  </oneCellAnchor>
-  <oneCellAnchor>
-    <from>
-      <col>5</col>
-      <colOff>0</colOff>
-      <row>61</row>
+        <cNvPr id="60" name="Image 60" descr="Picture"/>
+        <cNvPicPr/>
+      </nvPicPr>
+      <blipFill>
+        <a:blip cstate="print" r:embed="rId60"/>
+        <a:stretch>
+          <a:fillRect/>
+        </a:stretch>
+      </blipFill>
+      <spPr>
+        <a:prstGeom prst="rect"/>
+      </spPr>
+    </pic>
+    <clientData/>
+  </oneCellAnchor>
+  <oneCellAnchor>
+    <from>
+      <col>5</col>
+      <colOff>0</colOff>
+      <row>63</row>
       <rowOff>0</rowOff>
     </from>
     <ext cx="466725" cy="838200"/>
     <pic>
       <nvPicPr>
-        <cNvPr id="59" name="Image 59" descr="Picture"/>
-        <cNvPicPr/>
-      </nvPicPr>
-      <blipFill>
-        <a:blip cstate="print" r:embed="rId59"/>
-        <a:stretch>
-          <a:fillRect/>
-        </a:stretch>
-      </blipFill>
-      <spPr>
-        <a:prstGeom prst="rect"/>
-      </spPr>
-    </pic>
-    <clientData/>
-  </oneCellAnchor>
-  <oneCellAnchor>
-    <from>
-      <col>5</col>
-      <colOff>0</colOff>
-      <row>62</row>
+        <cNvPr id="61" name="Image 61" descr="Picture"/>
+        <cNvPicPr/>
+      </nvPicPr>
+      <blipFill>
+        <a:blip cstate="print" r:embed="rId61"/>
+        <a:stretch>
+          <a:fillRect/>
+        </a:stretch>
+      </blipFill>
+      <spPr>
+        <a:prstGeom prst="rect"/>
+      </spPr>
+    </pic>
+    <clientData/>
+  </oneCellAnchor>
+  <oneCellAnchor>
+    <from>
+      <col>5</col>
+      <colOff>0</colOff>
+      <row>64</row>
       <rowOff>0</rowOff>
     </from>
     <ext cx="733425" cy="838200"/>
     <pic>
       <nvPicPr>
-        <cNvPr id="60" name="Image 60" descr="Picture"/>
-        <cNvPicPr/>
-      </nvPicPr>
-      <blipFill>
-        <a:blip cstate="print" r:embed="rId60"/>
-        <a:stretch>
-          <a:fillRect/>
-        </a:stretch>
-      </blipFill>
-      <spPr>
-        <a:prstGeom prst="rect"/>
-      </spPr>
-    </pic>
-    <clientData/>
-  </oneCellAnchor>
-  <oneCellAnchor>
-    <from>
-      <col>5</col>
-      <colOff>0</colOff>
-      <row>63</row>
+        <cNvPr id="62" name="Image 62" descr="Picture"/>
+        <cNvPicPr/>
+      </nvPicPr>
+      <blipFill>
+        <a:blip cstate="print" r:embed="rId62"/>
+        <a:stretch>
+          <a:fillRect/>
+        </a:stretch>
+      </blipFill>
+      <spPr>
+        <a:prstGeom prst="rect"/>
+      </spPr>
+    </pic>
+    <clientData/>
+  </oneCellAnchor>
+  <oneCellAnchor>
+    <from>
+      <col>5</col>
+      <colOff>0</colOff>
+      <row>65</row>
       <rowOff>0</rowOff>
     </from>
     <ext cx="371475" cy="838200"/>
     <pic>
       <nvPicPr>
-        <cNvPr id="61" name="Image 61" descr="Picture"/>
-        <cNvPicPr/>
-      </nvPicPr>
-      <blipFill>
-        <a:blip cstate="print" r:embed="rId61"/>
-        <a:stretch>
-          <a:fillRect/>
-        </a:stretch>
-      </blipFill>
-      <spPr>
-        <a:prstGeom prst="rect"/>
-      </spPr>
-    </pic>
-    <clientData/>
-  </oneCellAnchor>
-  <oneCellAnchor>
-    <from>
-      <col>5</col>
-      <colOff>0</colOff>
-      <row>64</row>
+        <cNvPr id="63" name="Image 63" descr="Picture"/>
+        <cNvPicPr/>
+      </nvPicPr>
+      <blipFill>
+        <a:blip cstate="print" r:embed="rId63"/>
+        <a:stretch>
+          <a:fillRect/>
+        </a:stretch>
+      </blipFill>
+      <spPr>
+        <a:prstGeom prst="rect"/>
+      </spPr>
+    </pic>
+    <clientData/>
+  </oneCellAnchor>
+  <oneCellAnchor>
+    <from>
+      <col>5</col>
+      <colOff>0</colOff>
+      <row>66</row>
       <rowOff>0</rowOff>
     </from>
     <ext cx="466725" cy="838200"/>
     <pic>
       <nvPicPr>
-        <cNvPr id="62" name="Image 62" descr="Picture"/>
-        <cNvPicPr/>
-      </nvPicPr>
-      <blipFill>
-        <a:blip cstate="print" r:embed="rId62"/>
-        <a:stretch>
-          <a:fillRect/>
-        </a:stretch>
-      </blipFill>
-      <spPr>
-        <a:prstGeom prst="rect"/>
-      </spPr>
-    </pic>
-    <clientData/>
-  </oneCellAnchor>
-  <oneCellAnchor>
-    <from>
-      <col>5</col>
-      <colOff>0</colOff>
-      <row>65</row>
+        <cNvPr id="64" name="Image 64" descr="Picture"/>
+        <cNvPicPr/>
+      </nvPicPr>
+      <blipFill>
+        <a:blip cstate="print" r:embed="rId64"/>
+        <a:stretch>
+          <a:fillRect/>
+        </a:stretch>
+      </blipFill>
+      <spPr>
+        <a:prstGeom prst="rect"/>
+      </spPr>
+    </pic>
+    <clientData/>
+  </oneCellAnchor>
+  <oneCellAnchor>
+    <from>
+      <col>5</col>
+      <colOff>0</colOff>
+      <row>67</row>
       <rowOff>0</rowOff>
     </from>
     <ext cx="466725" cy="838200"/>
     <pic>
       <nvPicPr>
-        <cNvPr id="63" name="Image 63" descr="Picture"/>
-        <cNvPicPr/>
-      </nvPicPr>
-      <blipFill>
-        <a:blip cstate="print" r:embed="rId63"/>
-        <a:stretch>
-          <a:fillRect/>
-        </a:stretch>
-      </blipFill>
-      <spPr>
-        <a:prstGeom prst="rect"/>
-      </spPr>
-    </pic>
-    <clientData/>
-  </oneCellAnchor>
-  <oneCellAnchor>
-    <from>
-      <col>5</col>
-      <colOff>0</colOff>
-      <row>66</row>
+        <cNvPr id="65" name="Image 65" descr="Picture"/>
+        <cNvPicPr/>
+      </nvPicPr>
+      <blipFill>
+        <a:blip cstate="print" r:embed="rId65"/>
+        <a:stretch>
+          <a:fillRect/>
+        </a:stretch>
+      </blipFill>
+      <spPr>
+        <a:prstGeom prst="rect"/>
+      </spPr>
+    </pic>
+    <clientData/>
+  </oneCellAnchor>
+  <oneCellAnchor>
+    <from>
+      <col>5</col>
+      <colOff>0</colOff>
+      <row>68</row>
       <rowOff>0</rowOff>
     </from>
     <ext cx="466725" cy="838200"/>
     <pic>
       <nvPicPr>
-        <cNvPr id="64" name="Image 64" descr="Picture"/>
-        <cNvPicPr/>
-      </nvPicPr>
-      <blipFill>
-        <a:blip cstate="print" r:embed="rId64"/>
-        <a:stretch>
-          <a:fillRect/>
-        </a:stretch>
-      </blipFill>
-      <spPr>
-        <a:prstGeom prst="rect"/>
-      </spPr>
-    </pic>
-    <clientData/>
-  </oneCellAnchor>
-  <oneCellAnchor>
-    <from>
-      <col>5</col>
-      <colOff>0</colOff>
-      <row>67</row>
+        <cNvPr id="66" name="Image 66" descr="Picture"/>
+        <cNvPicPr/>
+      </nvPicPr>
+      <blipFill>
+        <a:blip cstate="print" r:embed="rId66"/>
+        <a:stretch>
+          <a:fillRect/>
+        </a:stretch>
+      </blipFill>
+      <spPr>
+        <a:prstGeom prst="rect"/>
+      </spPr>
+    </pic>
+    <clientData/>
+  </oneCellAnchor>
+  <oneCellAnchor>
+    <from>
+      <col>5</col>
+      <colOff>0</colOff>
+      <row>69</row>
       <rowOff>0</rowOff>
     </from>
     <ext cx="647700" cy="838200"/>
     <pic>
       <nvPicPr>
-        <cNvPr id="65" name="Image 65" descr="Picture"/>
-        <cNvPicPr/>
-      </nvPicPr>
-      <blipFill>
-        <a:blip cstate="print" r:embed="rId65"/>
+        <cNvPr id="67" name="Image 67" descr="Picture"/>
+        <cNvPicPr/>
+      </nvPicPr>
+      <blipFill>
+        <a:blip cstate="print" r:embed="rId67"/>
         <a:stretch>
           <a:fillRect/>
         </a:stretch>
@@ -2210,7 +2260,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:G68"/>
+  <dimension ref="A1:G70"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="14.45"/>
   <cols>
     <col width="7" customWidth="1" style="1" min="1" max="1"/>
@@ -2238,7 +2288,7 @@
     <row r="2" ht="20.1" customHeight="1">
       <c r="A2" s="8" t="inlineStr">
         <is>
-          <t>Total: 65 employees across 12 brands / departments   |   Brands: Bigg Bear, B2B, Eggspert, OG Pizza, Koby's, The Chatpata Affair, The Momo Box, Burrito Bros, The Coffee Vault, Maintenance Head, Crownest, Crownest Floor Manager</t>
+          <t>Total: 67 employees across 12 brands / departments   |   Brands: Bigg Bear, B2B, Eggspert, OG Pizza, Koby's, The Chatpata Affair, The Momo Box, Burrito Bros, The Coffee Vault, Maintenance Head, Crownest, Crownest Floor Manager</t>
         </is>
       </c>
       <c r="B2" s="10" t="n"/>
@@ -3456,33 +3506,21 @@
       </c>
     </row>
     <row r="42" ht="70" customHeight="1">
-      <c r="A42" s="14" t="n">
+      <c r="A42" s="12" t="n">
         <v>39</v>
       </c>
-      <c r="B42" s="14" t="inlineStr">
-        <is>
-          <t>Santosh Kumar</t>
-        </is>
-      </c>
-      <c r="C42" s="15" t="inlineStr">
-        <is>
-          <t>TCA-204</t>
-        </is>
-      </c>
-      <c r="D42" s="15" t="inlineStr">
-        <is>
-          <t>9305946728</t>
-        </is>
-      </c>
-      <c r="E42" s="15" t="inlineStr">
-        <is>
-          <t>6158 6990 5833</t>
-        </is>
-      </c>
-      <c r="F42" s="14" t="n"/>
-      <c r="G42" s="14" t="inlineStr">
-        <is>
-          <t>The Chatpata Affair</t>
+      <c r="B42" s="12" t="inlineStr">
+        <is>
+          <t>Pushpendra</t>
+        </is>
+      </c>
+      <c r="C42" s="13" t="n"/>
+      <c r="D42" s="13" t="n"/>
+      <c r="E42" s="13" t="n"/>
+      <c r="F42" s="12" t="n"/>
+      <c r="G42" s="12" t="inlineStr">
+        <is>
+          <t>Koby's</t>
         </is>
       </c>
     </row>
@@ -3492,22 +3530,22 @@
       </c>
       <c r="B43" s="14" t="inlineStr">
         <is>
-          <t>Gaurav Arya</t>
+          <t>Santosh Kumar</t>
         </is>
       </c>
       <c r="C43" s="15" t="inlineStr">
         <is>
-          <t>TCA-302</t>
+          <t>TCA-204</t>
         </is>
       </c>
       <c r="D43" s="15" t="inlineStr">
         <is>
-          <t>8006058432</t>
+          <t>9305946728</t>
         </is>
       </c>
       <c r="E43" s="15" t="inlineStr">
         <is>
-          <t>2354 4261 0569</t>
+          <t>6158 6990 5833</t>
         </is>
       </c>
       <c r="F43" s="14" t="n"/>
@@ -3523,22 +3561,22 @@
       </c>
       <c r="B44" s="14" t="inlineStr">
         <is>
-          <t>Narendra Kumar Arya</t>
+          <t>Gaurav Arya</t>
         </is>
       </c>
       <c r="C44" s="15" t="inlineStr">
         <is>
-          <t>TCA-207</t>
+          <t>TCA-302</t>
         </is>
       </c>
       <c r="D44" s="15" t="inlineStr">
         <is>
-          <t>9690999212</t>
+          <t>8006058432</t>
         </is>
       </c>
       <c r="E44" s="15" t="inlineStr">
         <is>
-          <t>2461 0635 8804</t>
+          <t>2354 4261 0569</t>
         </is>
       </c>
       <c r="F44" s="14" t="n"/>
@@ -3554,22 +3592,22 @@
       </c>
       <c r="B45" s="14" t="inlineStr">
         <is>
-          <t>Sahil</t>
+          <t>Narendra Kumar Arya</t>
         </is>
       </c>
       <c r="C45" s="15" t="inlineStr">
         <is>
-          <t>TCA-301</t>
+          <t>TCA-207</t>
         </is>
       </c>
       <c r="D45" s="15" t="inlineStr">
         <is>
-          <t>7070621218</t>
+          <t>9690999212</t>
         </is>
       </c>
       <c r="E45" s="15" t="inlineStr">
         <is>
-          <t>GHCPK3642K</t>
+          <t>2461 0635 8804</t>
         </is>
       </c>
       <c r="F45" s="14" t="n"/>
@@ -3585,22 +3623,22 @@
       </c>
       <c r="B46" s="14" t="inlineStr">
         <is>
-          <t>Himanshu</t>
+          <t>Sahil</t>
         </is>
       </c>
       <c r="C46" s="15" t="inlineStr">
         <is>
-          <t>TCA-321</t>
+          <t>TCA-301</t>
         </is>
       </c>
       <c r="D46" s="15" t="inlineStr">
         <is>
-          <t>+919044973472</t>
+          <t>7070621218</t>
         </is>
       </c>
       <c r="E46" s="15" t="inlineStr">
         <is>
-          <t>3308 4819 3577</t>
+          <t>GHCPK3642K</t>
         </is>
       </c>
       <c r="F46" s="14" t="n"/>
@@ -3611,33 +3649,33 @@
       </c>
     </row>
     <row r="47" ht="70" customHeight="1">
-      <c r="A47" s="12" t="n">
+      <c r="A47" s="14" t="n">
         <v>44</v>
       </c>
-      <c r="B47" s="12" t="inlineStr">
+      <c r="B47" s="14" t="inlineStr">
         <is>
           <t>Himanshu</t>
         </is>
       </c>
-      <c r="C47" s="13" t="inlineStr">
-        <is>
-          <t>MM-01</t>
-        </is>
-      </c>
-      <c r="D47" s="13" t="inlineStr">
-        <is>
-          <t>8130665709</t>
-        </is>
-      </c>
-      <c r="E47" s="13" t="inlineStr">
-        <is>
-          <t>5482 8020 7052</t>
-        </is>
-      </c>
-      <c r="F47" s="12" t="n"/>
-      <c r="G47" s="12" t="inlineStr">
-        <is>
-          <t>The Momo Box</t>
+      <c r="C47" s="15" t="inlineStr">
+        <is>
+          <t>TCA-321</t>
+        </is>
+      </c>
+      <c r="D47" s="15" t="inlineStr">
+        <is>
+          <t>+919044973472</t>
+        </is>
+      </c>
+      <c r="E47" s="15" t="inlineStr">
+        <is>
+          <t>3308 4819 3577</t>
+        </is>
+      </c>
+      <c r="F47" s="14" t="n"/>
+      <c r="G47" s="14" t="inlineStr">
+        <is>
+          <t>The Chatpata Affair</t>
         </is>
       </c>
     </row>
@@ -3647,22 +3685,22 @@
       </c>
       <c r="B48" s="12" t="inlineStr">
         <is>
-          <t>Ganesh Mehta</t>
+          <t>Himanshu</t>
         </is>
       </c>
       <c r="C48" s="13" t="inlineStr">
         <is>
-          <t>MM-06</t>
+          <t>MM-01</t>
         </is>
       </c>
       <c r="D48" s="13" t="inlineStr">
         <is>
-          <t>7535870127</t>
+          <t>8130665709</t>
         </is>
       </c>
       <c r="E48" s="13" t="inlineStr">
         <is>
-          <t>3571 5401 1548</t>
+          <t>5482 8020 7052</t>
         </is>
       </c>
       <c r="F48" s="12" t="n"/>
@@ -3678,18 +3716,22 @@
       </c>
       <c r="B49" s="12" t="inlineStr">
         <is>
-          <t>Gopal</t>
-        </is>
-      </c>
-      <c r="C49" s="13" t="n"/>
+          <t>Ganesh Mehta</t>
+        </is>
+      </c>
+      <c r="C49" s="13" t="inlineStr">
+        <is>
+          <t>MM-06</t>
+        </is>
+      </c>
       <c r="D49" s="13" t="inlineStr">
         <is>
-          <t>975965603</t>
+          <t>7535870127</t>
         </is>
       </c>
       <c r="E49" s="13" t="inlineStr">
         <is>
-          <t>2328 8290 9181</t>
+          <t>3571 5401 1548</t>
         </is>
       </c>
       <c r="F49" s="12" t="n"/>
@@ -3705,18 +3747,18 @@
       </c>
       <c r="B50" s="12" t="inlineStr">
         <is>
-          <t>Manas</t>
+          <t>Gopal</t>
         </is>
       </c>
       <c r="C50" s="13" t="n"/>
       <c r="D50" s="13" t="inlineStr">
         <is>
-          <t>9670870565</t>
+          <t>975965603</t>
         </is>
       </c>
       <c r="E50" s="13" t="inlineStr">
         <is>
-          <t>5014 7570 6569</t>
+          <t>2328 8290 9181</t>
         </is>
       </c>
       <c r="F50" s="12" t="n"/>
@@ -3732,18 +3774,18 @@
       </c>
       <c r="B51" s="12" t="inlineStr">
         <is>
-          <t>Sunil</t>
+          <t>Manas</t>
         </is>
       </c>
       <c r="C51" s="13" t="n"/>
       <c r="D51" s="13" t="inlineStr">
         <is>
-          <t>6280274213</t>
+          <t>9670870565</t>
         </is>
       </c>
       <c r="E51" s="13" t="inlineStr">
         <is>
-          <t>6461 0616 7060</t>
+          <t>5014 7570 6569</t>
         </is>
       </c>
       <c r="F51" s="12" t="n"/>
@@ -3754,64 +3796,48 @@
       </c>
     </row>
     <row r="52" ht="70" customHeight="1">
-      <c r="A52" s="14" t="n">
+      <c r="A52" s="12" t="n">
         <v>49</v>
       </c>
-      <c r="B52" s="14" t="inlineStr">
-        <is>
-          <t>Jatin Jhawar</t>
-        </is>
-      </c>
-      <c r="C52" s="15" t="inlineStr">
-        <is>
-          <t>BB01</t>
-        </is>
-      </c>
-      <c r="D52" s="15" t="inlineStr">
-        <is>
-          <t>6202282230</t>
-        </is>
-      </c>
-      <c r="E52" s="15" t="inlineStr">
-        <is>
-          <t>9588 8197 0484</t>
-        </is>
-      </c>
-      <c r="F52" s="14" t="n"/>
-      <c r="G52" s="14" t="inlineStr">
-        <is>
-          <t>Burrito Bros</t>
+      <c r="B52" s="12" t="inlineStr">
+        <is>
+          <t>Sunil</t>
+        </is>
+      </c>
+      <c r="C52" s="13" t="n"/>
+      <c r="D52" s="13" t="inlineStr">
+        <is>
+          <t>6280274213</t>
+        </is>
+      </c>
+      <c r="E52" s="13" t="inlineStr">
+        <is>
+          <t>6461 0616 7060</t>
+        </is>
+      </c>
+      <c r="F52" s="12" t="n"/>
+      <c r="G52" s="12" t="inlineStr">
+        <is>
+          <t>The Momo Box</t>
         </is>
       </c>
     </row>
     <row r="53" ht="70" customHeight="1">
-      <c r="A53" s="14" t="n">
+      <c r="A53" s="12" t="n">
         <v>50</v>
       </c>
-      <c r="B53" s="14" t="inlineStr">
-        <is>
-          <t>Keshav Jhawar</t>
-        </is>
-      </c>
-      <c r="C53" s="15" t="inlineStr">
-        <is>
-          <t>BB02</t>
-        </is>
-      </c>
-      <c r="D53" s="15" t="inlineStr">
-        <is>
-          <t>7762040281</t>
-        </is>
-      </c>
-      <c r="E53" s="15" t="inlineStr">
-        <is>
-          <t>6383 4826 6615</t>
-        </is>
-      </c>
-      <c r="F53" s="14" t="n"/>
-      <c r="G53" s="14" t="inlineStr">
-        <is>
-          <t>Burrito Bros</t>
+      <c r="B53" s="12" t="inlineStr">
+        <is>
+          <t>Ashish Arya</t>
+        </is>
+      </c>
+      <c r="C53" s="13" t="n"/>
+      <c r="D53" s="13" t="n"/>
+      <c r="E53" s="13" t="n"/>
+      <c r="F53" s="12" t="n"/>
+      <c r="G53" s="12" t="inlineStr">
+        <is>
+          <t>The Momo Box</t>
         </is>
       </c>
     </row>
@@ -3821,22 +3847,22 @@
       </c>
       <c r="B54" s="14" t="inlineStr">
         <is>
-          <t>Milan Subedi</t>
+          <t>Jatin Jhawar</t>
         </is>
       </c>
       <c r="C54" s="15" t="inlineStr">
         <is>
-          <t>BB03</t>
+          <t>BB01</t>
         </is>
       </c>
       <c r="D54" s="15" t="inlineStr">
         <is>
-          <t>7770872441</t>
+          <t>6202282230</t>
         </is>
       </c>
       <c r="E54" s="15" t="inlineStr">
         <is>
-          <t>9333 0098 4316</t>
+          <t>9588 8197 0484</t>
         </is>
       </c>
       <c r="F54" s="14" t="n"/>
@@ -3852,22 +3878,22 @@
       </c>
       <c r="B55" s="14" t="inlineStr">
         <is>
-          <t>Manoj</t>
+          <t>Keshav Jhawar</t>
         </is>
       </c>
       <c r="C55" s="15" t="inlineStr">
         <is>
-          <t>BB04</t>
+          <t>BB02</t>
         </is>
       </c>
       <c r="D55" s="15" t="inlineStr">
         <is>
-          <t>7668864718</t>
+          <t>7762040281</t>
         </is>
       </c>
       <c r="E55" s="15" t="inlineStr">
         <is>
-          <t>3821 2210 4800</t>
+          <t>6383 4826 6615</t>
         </is>
       </c>
       <c r="F55" s="14" t="n"/>
@@ -3878,64 +3904,64 @@
       </c>
     </row>
     <row r="56" ht="70" customHeight="1">
-      <c r="A56" s="12" t="n">
+      <c r="A56" s="14" t="n">
         <v>53</v>
       </c>
-      <c r="B56" s="12" t="inlineStr">
-        <is>
-          <t>Ravi Maurya</t>
-        </is>
-      </c>
-      <c r="C56" s="13" t="inlineStr">
-        <is>
-          <t>TCV-001</t>
-        </is>
-      </c>
-      <c r="D56" s="13" t="inlineStr">
-        <is>
-          <t>N/A</t>
-        </is>
-      </c>
-      <c r="E56" s="13" t="inlineStr">
-        <is>
-          <t>9191 0244 4041</t>
-        </is>
-      </c>
-      <c r="F56" s="12" t="n"/>
-      <c r="G56" s="12" t="inlineStr">
-        <is>
-          <t>The Coffee Vault</t>
+      <c r="B56" s="14" t="inlineStr">
+        <is>
+          <t>Milan Subedi</t>
+        </is>
+      </c>
+      <c r="C56" s="15" t="inlineStr">
+        <is>
+          <t>BB03</t>
+        </is>
+      </c>
+      <c r="D56" s="15" t="inlineStr">
+        <is>
+          <t>7770872441</t>
+        </is>
+      </c>
+      <c r="E56" s="15" t="inlineStr">
+        <is>
+          <t>9333 0098 4316</t>
+        </is>
+      </c>
+      <c r="F56" s="14" t="n"/>
+      <c r="G56" s="14" t="inlineStr">
+        <is>
+          <t>Burrito Bros</t>
         </is>
       </c>
     </row>
     <row r="57" ht="70" customHeight="1">
-      <c r="A57" s="12" t="n">
+      <c r="A57" s="14" t="n">
         <v>54</v>
       </c>
-      <c r="B57" s="12" t="inlineStr">
-        <is>
-          <t>Deepak Chauhan</t>
-        </is>
-      </c>
-      <c r="C57" s="13" t="inlineStr">
-        <is>
-          <t>TCV-002</t>
-        </is>
-      </c>
-      <c r="D57" s="13" t="inlineStr">
-        <is>
-          <t>+91 75055 56049</t>
-        </is>
-      </c>
-      <c r="E57" s="13" t="inlineStr">
-        <is>
-          <t>7416 5082 4706</t>
-        </is>
-      </c>
-      <c r="F57" s="12" t="n"/>
-      <c r="G57" s="12" t="inlineStr">
-        <is>
-          <t>The Coffee Vault</t>
+      <c r="B57" s="14" t="inlineStr">
+        <is>
+          <t>Manoj</t>
+        </is>
+      </c>
+      <c r="C57" s="15" t="inlineStr">
+        <is>
+          <t>BB04</t>
+        </is>
+      </c>
+      <c r="D57" s="15" t="inlineStr">
+        <is>
+          <t>7668864718</t>
+        </is>
+      </c>
+      <c r="E57" s="15" t="inlineStr">
+        <is>
+          <t>3821 2210 4800</t>
+        </is>
+      </c>
+      <c r="F57" s="14" t="n"/>
+      <c r="G57" s="14" t="inlineStr">
+        <is>
+          <t>Burrito Bros</t>
         </is>
       </c>
     </row>
@@ -3945,22 +3971,22 @@
       </c>
       <c r="B58" s="12" t="inlineStr">
         <is>
-          <t>Sunny</t>
+          <t>Ravi Maurya</t>
         </is>
       </c>
       <c r="C58" s="13" t="inlineStr">
         <is>
-          <t>TCV-003</t>
+          <t>TCV-001</t>
         </is>
       </c>
       <c r="D58" s="13" t="inlineStr">
         <is>
-          <t>+91 99537 65782</t>
+          <t>N/A</t>
         </is>
       </c>
       <c r="E58" s="13" t="inlineStr">
         <is>
-          <t>6665 2709 5607</t>
+          <t>9191 0244 4041</t>
         </is>
       </c>
       <c r="F58" s="12" t="n"/>
@@ -3976,22 +4002,22 @@
       </c>
       <c r="B59" s="12" t="inlineStr">
         <is>
-          <t>Sandeep Shriwas</t>
+          <t>Deepak Chauhan</t>
         </is>
       </c>
       <c r="C59" s="13" t="inlineStr">
         <is>
-          <t>TCV-004</t>
+          <t>TCV-002</t>
         </is>
       </c>
       <c r="D59" s="13" t="inlineStr">
         <is>
-          <t>N/A</t>
+          <t>+91 75055 56049</t>
         </is>
       </c>
       <c r="E59" s="13" t="inlineStr">
         <is>
-          <t>4695 8962 0647</t>
+          <t>7416 5082 4706</t>
         </is>
       </c>
       <c r="F59" s="12" t="n"/>
@@ -4007,22 +4033,22 @@
       </c>
       <c r="B60" s="12" t="inlineStr">
         <is>
-          <t>Sunil Kushwaha</t>
+          <t>Sunny</t>
         </is>
       </c>
       <c r="C60" s="13" t="inlineStr">
         <is>
-          <t>TCV-005</t>
+          <t>TCV-003</t>
         </is>
       </c>
       <c r="D60" s="13" t="inlineStr">
         <is>
-          <t>+91 82698 80641</t>
+          <t>+91 99537 65782</t>
         </is>
       </c>
       <c r="E60" s="13" t="inlineStr">
         <is>
-          <t>4885 3404 7284</t>
+          <t>6665 2709 5607</t>
         </is>
       </c>
       <c r="F60" s="12" t="n"/>
@@ -4033,33 +4059,33 @@
       </c>
     </row>
     <row r="61" ht="70" customHeight="1">
-      <c r="A61" s="14" t="n">
+      <c r="A61" s="12" t="n">
         <v>58</v>
       </c>
-      <c r="B61" s="14" t="inlineStr">
-        <is>
-          <t>Dharminder Singh</t>
-        </is>
-      </c>
-      <c r="C61" s="15" t="inlineStr">
-        <is>
-          <t>005</t>
-        </is>
-      </c>
-      <c r="D61" s="15" t="inlineStr">
-        <is>
-          <t>+91 99589 13516</t>
-        </is>
-      </c>
-      <c r="E61" s="15" t="inlineStr">
-        <is>
-          <t>6730 3995 5245</t>
-        </is>
-      </c>
-      <c r="F61" s="14" t="n"/>
-      <c r="G61" s="14" t="inlineStr">
-        <is>
-          <t>Maintenance Head</t>
+      <c r="B61" s="12" t="inlineStr">
+        <is>
+          <t>Sandeep Shriwas</t>
+        </is>
+      </c>
+      <c r="C61" s="13" t="inlineStr">
+        <is>
+          <t>TCV-004</t>
+        </is>
+      </c>
+      <c r="D61" s="13" t="inlineStr">
+        <is>
+          <t>N/A</t>
+        </is>
+      </c>
+      <c r="E61" s="13" t="inlineStr">
+        <is>
+          <t>4695 8962 0647</t>
+        </is>
+      </c>
+      <c r="F61" s="12" t="n"/>
+      <c r="G61" s="12" t="inlineStr">
+        <is>
+          <t>The Coffee Vault</t>
         </is>
       </c>
     </row>
@@ -4069,55 +4095,59 @@
       </c>
       <c r="B62" s="12" t="inlineStr">
         <is>
-          <t>Pawan Rajput</t>
+          <t>Sunil Kushwaha</t>
         </is>
       </c>
       <c r="C62" s="13" t="inlineStr">
         <is>
-          <t>CN01</t>
+          <t>TCV-005</t>
         </is>
       </c>
       <c r="D62" s="13" t="inlineStr">
         <is>
-          <t>9560464601</t>
+          <t>+91 82698 80641</t>
         </is>
       </c>
       <c r="E62" s="13" t="inlineStr">
         <is>
-          <t>7211 9046 7109</t>
+          <t>4885 3404 7284</t>
         </is>
       </c>
       <c r="F62" s="12" t="n"/>
       <c r="G62" s="12" t="inlineStr">
         <is>
-          <t>Crownest</t>
+          <t>The Coffee Vault</t>
         </is>
       </c>
     </row>
     <row r="63" ht="70" customFormat="1" customHeight="1" s="2">
-      <c r="A63" s="12" t="n">
+      <c r="A63" s="14" t="n">
         <v>60</v>
       </c>
-      <c r="B63" s="12" t="inlineStr">
-        <is>
-          <t>Sunny Gupta</t>
-        </is>
-      </c>
-      <c r="C63" s="13" t="inlineStr">
-        <is>
-          <t>CN07</t>
-        </is>
-      </c>
-      <c r="D63" s="13" t="inlineStr">
-        <is>
-          <t>+91 92056 54232</t>
-        </is>
-      </c>
-      <c r="E63" s="13" t="n"/>
-      <c r="F63" s="12" t="n"/>
-      <c r="G63" s="12" t="inlineStr">
-        <is>
-          <t>Crownest</t>
+      <c r="B63" s="14" t="inlineStr">
+        <is>
+          <t>Dharminder Singh</t>
+        </is>
+      </c>
+      <c r="C63" s="15" t="inlineStr">
+        <is>
+          <t>005</t>
+        </is>
+      </c>
+      <c r="D63" s="15" t="inlineStr">
+        <is>
+          <t>+91 99589 13516</t>
+        </is>
+      </c>
+      <c r="E63" s="15" t="inlineStr">
+        <is>
+          <t>6730 3995 5245</t>
+        </is>
+      </c>
+      <c r="F63" s="14" t="n"/>
+      <c r="G63" s="14" t="inlineStr">
+        <is>
+          <t>Maintenance Head</t>
         </is>
       </c>
     </row>
@@ -4127,22 +4157,22 @@
       </c>
       <c r="B64" s="12" t="inlineStr">
         <is>
-          <t>Vansh</t>
+          <t>Pawan Rajput</t>
         </is>
       </c>
       <c r="C64" s="13" t="inlineStr">
         <is>
-          <t>CN02</t>
+          <t>CN01</t>
         </is>
       </c>
       <c r="D64" s="13" t="inlineStr">
         <is>
-          <t>+91 92172 58511</t>
+          <t>9560464601</t>
         </is>
       </c>
       <c r="E64" s="13" t="inlineStr">
         <is>
-          <t>3193 2738 9222</t>
+          <t>7211 9046 7109</t>
         </is>
       </c>
       <c r="F64" s="12" t="n"/>
@@ -4158,24 +4188,20 @@
       </c>
       <c r="B65" s="12" t="inlineStr">
         <is>
-          <t>Ashish Kumar</t>
+          <t>Sunny Gupta</t>
         </is>
       </c>
       <c r="C65" s="13" t="inlineStr">
         <is>
-          <t>CN03</t>
+          <t>CN07</t>
         </is>
       </c>
       <c r="D65" s="13" t="inlineStr">
         <is>
-          <t>+91 97185 61709</t>
-        </is>
-      </c>
-      <c r="E65" s="13" t="inlineStr">
-        <is>
-          <t>7780 4640 0298</t>
-        </is>
-      </c>
+          <t>+91 92056 54232</t>
+        </is>
+      </c>
+      <c r="E65" s="13" t="n"/>
       <c r="F65" s="12" t="n"/>
       <c r="G65" s="12" t="inlineStr">
         <is>
@@ -4189,22 +4215,22 @@
       </c>
       <c r="B66" s="12" t="inlineStr">
         <is>
-          <t>Yesh Kumar</t>
+          <t>Vansh</t>
         </is>
       </c>
       <c r="C66" s="13" t="inlineStr">
         <is>
-          <t>CN04</t>
+          <t>CN02</t>
         </is>
       </c>
       <c r="D66" s="13" t="inlineStr">
         <is>
-          <t>+91 88262 56951</t>
+          <t>+91 92172 58511</t>
         </is>
       </c>
       <c r="E66" s="13" t="inlineStr">
         <is>
-          <t>9811 9163 4774</t>
+          <t>3193 2738 9222</t>
         </is>
       </c>
       <c r="F66" s="12" t="n"/>
@@ -4220,22 +4246,22 @@
       </c>
       <c r="B67" s="12" t="inlineStr">
         <is>
-          <t>Manjeet Kumar</t>
+          <t>Ashish Kumar</t>
         </is>
       </c>
       <c r="C67" s="13" t="inlineStr">
         <is>
-          <t>CN05</t>
+          <t>CN03</t>
         </is>
       </c>
       <c r="D67" s="13" t="inlineStr">
         <is>
-          <t>+91 63961 15541</t>
+          <t>+91 97185 61709</t>
         </is>
       </c>
       <c r="E67" s="13" t="inlineStr">
         <is>
-          <t>6585 1587 2218</t>
+          <t>7780 4640 0298</t>
         </is>
       </c>
       <c r="F67" s="12" t="n"/>
@@ -4246,38 +4272,98 @@
       </c>
     </row>
     <row r="68" ht="70" customFormat="1" customHeight="1" s="2">
-      <c r="A68" s="14" t="n">
+      <c r="A68" s="12" t="n">
         <v>65</v>
       </c>
-      <c r="B68" s="14" t="inlineStr">
+      <c r="B68" s="12" t="inlineStr">
+        <is>
+          <t>Yesh Kumar</t>
+        </is>
+      </c>
+      <c r="C68" s="13" t="inlineStr">
+        <is>
+          <t>CN04</t>
+        </is>
+      </c>
+      <c r="D68" s="13" t="inlineStr">
+        <is>
+          <t>+91 88262 56951</t>
+        </is>
+      </c>
+      <c r="E68" s="13" t="inlineStr">
+        <is>
+          <t>9811 9163 4774</t>
+        </is>
+      </c>
+      <c r="F68" s="12" t="n"/>
+      <c r="G68" s="12" t="inlineStr">
+        <is>
+          <t>Crownest</t>
+        </is>
+      </c>
+    </row>
+    <row r="69" ht="70" customFormat="1" customHeight="1" s="2">
+      <c r="A69" s="12" t="n">
+        <v>66</v>
+      </c>
+      <c r="B69" s="12" t="inlineStr">
+        <is>
+          <t>Manjeet Kumar</t>
+        </is>
+      </c>
+      <c r="C69" s="13" t="inlineStr">
+        <is>
+          <t>CN05</t>
+        </is>
+      </c>
+      <c r="D69" s="13" t="inlineStr">
+        <is>
+          <t>+91 63961 15541</t>
+        </is>
+      </c>
+      <c r="E69" s="13" t="inlineStr">
+        <is>
+          <t>6585 1587 2218</t>
+        </is>
+      </c>
+      <c r="F69" s="12" t="n"/>
+      <c r="G69" s="12" t="inlineStr">
+        <is>
+          <t>Crownest</t>
+        </is>
+      </c>
+    </row>
+    <row r="70" ht="70" customFormat="1" customHeight="1" s="2">
+      <c r="A70" s="14" t="n">
+        <v>67</v>
+      </c>
+      <c r="B70" s="14" t="inlineStr">
         <is>
           <t>Nitish Kumar Mishra</t>
         </is>
       </c>
-      <c r="C68" s="15" t="inlineStr">
+      <c r="C70" s="15" t="inlineStr">
         <is>
           <t>CN06</t>
         </is>
       </c>
-      <c r="D68" s="15" t="inlineStr">
+      <c r="D70" s="15" t="inlineStr">
         <is>
           <t>8810289632</t>
         </is>
       </c>
-      <c r="E68" s="15" t="inlineStr">
+      <c r="E70" s="15" t="inlineStr">
         <is>
           <t>6497 4797 9710</t>
         </is>
       </c>
-      <c r="F68" s="14" t="n"/>
-      <c r="G68" s="14" t="inlineStr">
+      <c r="F70" s="14" t="n"/>
+      <c r="G70" s="14" t="inlineStr">
         <is>
           <t>Crownest Floor Manager</t>
         </is>
       </c>
     </row>
-    <row r="69" ht="69.95" customFormat="1" customHeight="1" s="2"/>
-    <row r="70" ht="69.95" customFormat="1" customHeight="1" s="2"/>
     <row r="71" ht="69.95" customFormat="1" customHeight="1" s="2"/>
     <row r="72" ht="69.95" customFormat="1" customHeight="1" s="2"/>
     <row r="73" ht="60.95" customFormat="1" customHeight="1" s="2"/>

</xml_diff>